<commit_message>
Complete MEDIAN v0.5.0 Gate 4 hardening
</commit_message>
<xml_diff>
--- a/m050/extraction/progress/M050_Compile_Progress_and_Stage_Guide_v0_1_MEDIANv0_5_0.xlsx
+++ b/m050/extraction/progress/M050_Compile_Progress_and_Stage_Guide_v0_1_MEDIANv0_5_0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress &amp; Stages" sheetId="1" r:id="R4efdf136e1fe4b77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress &amp; Stages" sheetId="1" r:id="Re97e3e605248415e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -264,7 +264,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -275,7 +275,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -285,7 +285,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -296,7 +296,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +306,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -316,7 +316,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -326,7 +326,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -336,7 +336,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -346,7 +346,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -357,7 +357,7 @@
         <x:color rgb="FF9A2E2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9DDDD"/>
         </x:patternFill>
       </x:fill>
@@ -368,7 +368,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -379,7 +379,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -389,7 +389,7 @@
         <x:color rgb="FF176238"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCEFE2"/>
         </x:patternFill>
       </x:fill>
@@ -400,7 +400,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +410,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -420,7 +420,7 @@
         <x:color rgb="FF7A5200"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -430,7 +430,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -440,7 +440,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -450,7 +450,7 @@
         <x:color rgb="FF4C5967"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE9EDF1"/>
         </x:patternFill>
       </x:fill>
@@ -461,7 +461,7 @@
         <x:color rgb="FF9A2E2E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF9DDDD"/>
         </x:patternFill>
       </x:fill>
@@ -729,7 +729,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>Current state after Gates 1–3 and the ongoing Gate 4 cleanup. Costs are intentionally excluded and remain under m050/docs/operations/costs.</x:v>
+        <x:v>Current state after Gate 4 completion. Costs are intentionally excluded and remain in the dedicated Markdown ledger.</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
         <x:v>Current state after Gates 1–3 and the ongoing Gate 4 cleanup. Costs are intentionally excluded and remain under m050/docs/operations/costs.</x:v>
@@ -781,7 +781,7 @@
         <x:v>Current control gate</x:v>
       </x:c>
       <x:c r="B5" s="33" t="str">
-        <x:v>Gate 4 — source identity and drift retirement</x:v>
+        <x:v>Gate 4 complete; Gate 5 not begun</x:v>
       </x:c>
       <x:c r="C5" s="29"/>
       <x:c r="D5" s="32" t="str">
@@ -789,7 +789,7 @@
       </x:c>
       <x:c r="E5" s="33" t="n">
         <x:f>COUNTIF(D11:D15,"Complete")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="29"/>
       <x:c r="G5" s="29"/>
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="E6" s="35" t="n">
         <x:f>COUNTIF(D11:D15,"In progress")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="29"/>
       <x:c r="G6" s="29"/>
@@ -824,7 +824,7 @@
         <x:v>Next controlling decision</x:v>
       </x:c>
       <x:c r="E7" s="37" t="str">
-        <x:v>Finish Gate 4, then specify and verify Gate 5 implementation</x:v>
+        <x:v>Design and review Gate 5 extraction architecture; no provider calls</x:v>
       </x:c>
       <x:c r="F7" s="29"/>
       <x:c r="G7" s="29"/>
@@ -964,16 +964,16 @@
         <x:v>Correct misleading names and retire drift-era controls and run artifacts.</x:v>
       </x:c>
       <x:c r="D14" s="40" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="E14" s="40" t="str">
-        <x:v>Renames and archival substantially complete</x:v>
+        <x:v>Gate 4 completion report and receipt</x:v>
       </x:c>
       <x:c r="F14" s="40" t="str">
-        <x:v>Final validation and completion receipt</x:v>
+        <x:v>Frozen corpus, clean active tree, guard passes</x:v>
       </x:c>
       <x:c r="G14" s="40" t="str">
-        <x:v>Finish repository-wide checks and tracker refresh</x:v>
+        <x:v>Proceed to Gate 5 design discussion</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1294,8 +1294,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd66b46435804ce1"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9507ef0dcd404a2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd7fbab436f40cb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3301eb872524e3e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Build Gate 5 offline processing foundation
</commit_message>
<xml_diff>
--- a/m050/extraction/progress/M050_Compile_Progress_and_Stage_Guide_v0_1_MEDIANv0_5_0.xlsx
+++ b/m050/extraction/progress/M050_Compile_Progress_and_Stage_Guide_v0_1_MEDIANv0_5_0.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress &amp; Stages" sheetId="1" r:id="Re97e3e605248415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progress &amp; Stages" sheetId="1" r:id="R9d5c8468960f4899"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -729,7 +729,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="28" t="str">
-        <x:v>Current state after Gate 4 completion. Costs are intentionally excluded and remain in the dedicated Markdown ledger.</x:v>
+        <x:v>Current Gate 5 offline-foundation state. Costs remain in the dedicated Markdown ledger; provider calls remain unauthorized.</x:v>
       </x:c>
       <x:c r="B2" s="28" t="str">
         <x:v>Current state after Gates 1–3 and the ongoing Gate 4 cleanup. Costs are intentionally excluded and remain under m050/docs/operations/costs.</x:v>
@@ -781,7 +781,7 @@
         <x:v>Current control gate</x:v>
       </x:c>
       <x:c r="B5" s="33" t="str">
-        <x:v>Gate 4 complete; Gate 5 not begun</x:v>
+        <x:v>Gate 5 in progress — offline foundation verified</x:v>
       </x:c>
       <x:c r="C5" s="29"/>
       <x:c r="D5" s="32" t="str">
@@ -807,7 +807,7 @@
       </x:c>
       <x:c r="E6" s="35" t="n">
         <x:f>COUNTIF(D11:D15,"In progress")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F6" s="29"/>
       <x:c r="G6" s="29"/>
@@ -817,14 +817,14 @@
         <x:v>External model calls</x:v>
       </x:c>
       <x:c r="B7" s="37" t="str">
-        <x:v>Frozen until Gate 5 implementation and dry-run verification</x:v>
+        <x:v>No provider calls; offline implementation and replay only</x:v>
       </x:c>
       <x:c r="C7" s="29"/>
       <x:c r="D7" s="36" t="str">
         <x:v>Next controlling decision</x:v>
       </x:c>
       <x:c r="E7" s="37" t="str">
-        <x:v>Design and review Gate 5 extraction architecture; no provider calls</x:v>
+        <x:v>Integrate controls and prepare deterministic legacy replay; no provider calls</x:v>
       </x:c>
       <x:c r="F7" s="29"/>
       <x:c r="G7" s="29"/>
@@ -987,16 +987,16 @@
         <x:v>Build the simpler source-bounded extraction system and prove it offline.</x:v>
       </x:c>
       <x:c r="D15" s="40" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="E15" s="40" t="str">
-        <x:v>No active runner yet</x:v>
+        <x:v>Approved technical contract; locked Mini runtime; 53-test offline foundation</x:v>
       </x:c>
       <x:c r="F15" s="40" t="str">
         <x:v>Verified dry run and controlled calibration approval</x:v>
       </x:c>
       <x:c r="G15" s="40" t="str">
-        <x:v>Begin only after Gate 4 passes</x:v>
+        <x:v>Integrate controls, then migrate reusable evidence offline</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1068,13 +1068,13 @@
         <x:v>No model</x:v>
       </x:c>
       <x:c r="E19" s="40" t="str">
-        <x:v>Pending Gate 5 implementation</x:v>
+        <x:v>Foundation implemented; source identity cards pending</x:v>
       </x:c>
       <x:c r="F19" s="40" t="str">
         <x:v>Every work order passes the identity gate</x:v>
       </x:c>
       <x:c r="G19" s="40" t="str">
-        <x:v>Implement manifest validation</x:v>
+        <x:v>Issue versioned identity cards and zero-call work orders</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1091,13 +1091,13 @@
         <x:v>No model</x:v>
       </x:c>
       <x:c r="E20" s="40" t="str">
-        <x:v>Pending Gate 5 implementation</x:v>
+        <x:v>Block and dual-limit chunk engine implemented and tested</x:v>
       </x:c>
       <x:c r="F20" s="40" t="str">
         <x:v>Complete block ledger and dry-run chunk plan</x:v>
       </x:c>
       <x:c r="G20" s="40" t="str">
-        <x:v>Implement block and dual-bound chunk controls</x:v>
+        <x:v>Run approved dry plans per source</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1137,13 +1137,13 @@
         <x:v>Deterministic + semantic review</x:v>
       </x:c>
       <x:c r="E22" s="40" t="str">
-        <x:v>Legacy evidence audited; new system not implemented</x:v>
+        <x:v>Validator implemented; semantic review workflow pending</x:v>
       </x:c>
       <x:c r="F22" s="40" t="str">
         <x:v>Accepted source evidence with receipts</x:v>
       </x:c>
       <x:c r="G22" s="40" t="str">
-        <x:v>Build validator and acceptance reports</x:v>
+        <x:v>Exercise legacy replay and review bundles</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1160,13 +1160,13 @@
         <x:v>Mapping layer</x:v>
       </x:c>
       <x:c r="E23" s="40" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Schema and validation foundation only; not authorized</x:v>
       </x:c>
       <x:c r="F23" s="40" t="str">
         <x:v>Every atom mapped, ambiguous, unmapped, invalid, or human-required</x:v>
       </x:c>
       <x:c r="G23" s="40" t="str">
-        <x:v>Start only after accepted evidence exists</x:v>
+        <x:v>Begin only after Layer E acceptance</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1183,13 +1183,13 @@
         <x:v>Cross-source review</x:v>
       </x:c>
       <x:c r="E24" s="40" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Bundle completeness foundation only; not authorized</x:v>
       </x:c>
       <x:c r="F24" s="40" t="str">
         <x:v>Every substantive atom has an explicit disposition</x:v>
       </x:c>
       <x:c r="G24" s="40" t="str">
-        <x:v>Do not begin during extraction</x:v>
+        <x:v>Calibrate only after Layer M is accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1294,8 +1294,8 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dd7fbab436f40cb"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3301eb872524e3e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac8c810407ca462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf0f67ace34f4325"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>